<commit_message>
Update Oct 05 outputs
</commit_message>
<xml_diff>
--- a/Oct - 05/Evening/Evening_OOS_Summary_2026-10-05.xlsx
+++ b/Oct - 05/Evening/Evening_OOS_Summary_2026-10-05.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -542,12 +542,12 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Total Outlets: 16</t>
+          <t>Total Outlets: 21</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Still OUT: 31</t>
+          <t>Still OUT: 34</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
@@ -890,43 +890,49 @@
       <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>KA-BLR-Cloud FC Malleshwaram</t>
+          <t>KA-BLR-Cloud FC Basaveshwara Nagar</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Assorted Cheesecakes (Pack Of 6)</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
+          <t>Assorted French Macarons (Pack Of 5)</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="inlineStr"/>
+      <c r="A15" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="9" t="inlineStr"/>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Cloud FC Electronic City</t>
+        </is>
+      </c>
       <c r="E15" s="5" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
+          <t>Signature Belgium Chocolate Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
         </is>
       </c>
     </row>
@@ -940,68 +946,68 @@
       <c r="C16" s="4" t="inlineStr"/>
       <c r="D16" s="9" t="inlineStr"/>
       <c r="E16" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="inlineStr">
+          <t>Danish Hazelnut Chocolate Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="4" t="inlineStr"/>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="9" t="inlineStr"/>
+      <c r="E17" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Pack Of 4 Medoviks And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Cloud FC Malleshwaram</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Cloud FC NBL</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Medoviks And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="9" t="inlineStr"/>
-      <c r="E18" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
         </is>
       </c>
     </row>
@@ -1015,16 +1021,16 @@
       <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" s="9" t="inlineStr"/>
       <c r="E19" s="5" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 5)</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Italian Tiramisu Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -1038,22 +1044,22 @@
       <c r="C20" s="4" t="inlineStr"/>
       <c r="D20" s="9" t="inlineStr"/>
       <c r="E20" s="5" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
@@ -1063,15 +1069,15 @@
       <c r="C21" s="4" t="inlineStr"/>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>KA-BLR-Cloud FC Whitefield</t>
+          <t>KA-BLR-Cloud FC NBL</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
+          <t>Pack Of 4 Medoviks And 4 Macarons</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -1081,31 +1087,25 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="4" t="n">
-        <v>7</v>
-      </c>
+      <c r="A22" s="4" t="inlineStr"/>
       <c r="B22" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Ivory Lounge JP Nagar</t>
-        </is>
-      </c>
+      <c r="D22" s="9" t="inlineStr"/>
       <c r="E22" s="5" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 5)</t>
-        </is>
-      </c>
-      <c r="G22" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
         </is>
       </c>
     </row>
@@ -1119,147 +1119,153 @@
       <c r="C23" s="4" t="inlineStr"/>
       <c r="D23" s="9" t="inlineStr"/>
       <c r="E23" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 5)</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" s="9" t="inlineStr"/>
+      <c r="E24" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Cloud FC Sarjapur</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Ivory Lounge JP Nagar</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 5)</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" s="9" t="inlineStr"/>
+      <c r="E27" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Assorted French Macarons (Pack Of 12)</t>
         </is>
       </c>
-      <c r="G23" s="10" t="inlineStr">
+      <c r="G27" s="10" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="4" t="n">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>HYD</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>TG-HYD-Cloud FC Attapur</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>HYD</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Cloud FC Attapur</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>Assorted Cheesecakes (Pack Of 6)</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="4" t="inlineStr"/>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr"/>
-      <c r="D25" s="9" t="inlineStr"/>
-      <c r="E25" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F28" s="7" t="inlineStr">
         <is>
           <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="4" t="inlineStr"/>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="9" t="inlineStr"/>
-      <c r="E26" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Lotus Biscoff Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr"/>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Cloud FC Charminar</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G27" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="4" t="inlineStr"/>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="9" t="inlineStr"/>
-      <c r="E28" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G28" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
         </is>
       </c>
     </row>
@@ -1273,68 +1279,68 @@
       <c r="C29" s="4" t="inlineStr"/>
       <c r="D29" s="9" t="inlineStr"/>
       <c r="E29" s="5" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
           <t>Lotus Biscoff Cheesecake With Macaron</t>
         </is>
       </c>
-      <c r="G29" s="10" t="inlineStr">
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr"/>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>TG-HYD-Cloud FC Charminar</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="4" t="inlineStr"/>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="9" t="inlineStr"/>
-      <c r="E30" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>Assorted Cheesecakes (Pack Of 12)</t>
-        </is>
-      </c>
-      <c r="G30" s="10" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="4" t="inlineStr"/>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr"/>
+      <c r="D31" s="9" t="inlineStr"/>
+      <c r="E31" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
         <is>
           <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Cloud FC Habsiguda</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
         </is>
       </c>
     </row>
@@ -1348,16 +1354,16 @@
       <c r="C32" s="4" t="inlineStr"/>
       <c r="D32" s="9" t="inlineStr"/>
       <c r="E32" s="5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Assorted Cheesecakes (Pack Of 6)</t>
-        </is>
-      </c>
-      <c r="G32" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Lotus Biscoff Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -1371,22 +1377,22 @@
       <c r="C33" s="4" t="inlineStr"/>
       <c r="D33" s="9" t="inlineStr"/>
       <c r="E33" s="5" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G33" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Assorted Cheesecakes (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
@@ -1396,101 +1402,95 @@
       <c r="C34" s="4" t="inlineStr"/>
       <c r="D34" s="6" t="inlineStr">
         <is>
+          <t>TG-HYD-Cloud FC Habsiguda</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="4" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr"/>
+      <c r="D35" s="9" t="inlineStr"/>
+      <c r="E35" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="4" t="inlineStr"/>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr"/>
+      <c r="D36" s="9" t="inlineStr"/>
+      <c r="E36" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
           <t>TG-HYD-Express Outlet Madhapur</t>
         </is>
       </c>
-      <c r="E34" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
-        </is>
-      </c>
-      <c r="G34" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Express Outlet Manikonda</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G35" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr"/>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Express Outlet Sainikpuri</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
-        </is>
-      </c>
-      <c r="G36" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="4" t="inlineStr"/>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr"/>
-      <c r="D37" s="9" t="inlineStr"/>
       <c r="E37" s="5" t="n">
         <v>19</v>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G37" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Italian Tiramisu Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -1503,22 +1503,18 @@
           <t>2026/10/05</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>MUM</t>
-        </is>
-      </c>
+      <c r="C38" s="4" t="inlineStr"/>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>MH-MUM-Cloud FC Borivali</t>
+          <t>TG-HYD-Express Outlet Manikonda</t>
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>Pack Of 4 Medoviks And 4 Macarons</t>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
@@ -1528,20 +1524,26 @@
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="4" t="inlineStr"/>
+      <c r="A39" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr"/>
-      <c r="D39" s="9" t="inlineStr"/>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>TG-HYD-Express Outlet Sainikpuri</t>
+        </is>
+      </c>
       <c r="E39" s="5" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 5)</t>
+          <t>Assorted French Macarons (Pack Of 12)</t>
         </is>
       </c>
       <c r="G39" s="8" t="inlineStr">
@@ -1560,11 +1562,11 @@
       <c r="C40" s="4" t="inlineStr"/>
       <c r="D40" s="9" t="inlineStr"/>
       <c r="E40" s="5" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -1574,20 +1576,30 @@
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="4" t="inlineStr"/>
+      <c r="A41" s="4" t="n">
+        <v>16</v>
+      </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr"/>
-      <c r="D41" s="9" t="inlineStr"/>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>MUM</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>MH-MUM-Cloud FC BKC</t>
+        </is>
+      </c>
       <c r="E41" s="5" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Signature Belgium Chocolate Medovik With Macaron</t>
+          <t>Assorted French Macarons (Pack Of 24)</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
@@ -1597,20 +1609,26 @@
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="4" t="inlineStr"/>
+      <c r="A42" s="4" t="n">
+        <v>17</v>
+      </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr"/>
-      <c r="D42" s="9" t="inlineStr"/>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>MH-MUM-Cloud FC Borivali</t>
+        </is>
+      </c>
       <c r="E42" s="5" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
+          <t>Assorted French Macarons (Pack Of 5)</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
@@ -1629,11 +1647,11 @@
       <c r="C43" s="4" t="inlineStr"/>
       <c r="D43" s="9" t="inlineStr"/>
       <c r="E43" s="5" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Danish Hazelnut Chocolate Medovik With Macaron</t>
+          <t>Assorted French Macarons (Pack Of 12)</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
@@ -1643,20 +1661,26 @@
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="4" t="inlineStr"/>
+      <c r="A44" s="4" t="n">
+        <v>18</v>
+      </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr"/>
-      <c r="D44" s="9" t="inlineStr"/>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>MH-MUM-Cloud FC Chembur</t>
+        </is>
+      </c>
       <c r="E44" s="5" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+          <t>Assorted French Macarons (Pack Of 5)</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
@@ -1675,11 +1699,11 @@
       <c r="C45" s="4" t="inlineStr"/>
       <c r="D45" s="9" t="inlineStr"/>
       <c r="E45" s="5" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Harley's Spl. Classic Russian Medovik With Macaron</t>
+          <t>Assorted French Macarons (Pack Of 12)</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
@@ -1698,76 +1722,151 @@
       <c r="C46" s="4" t="inlineStr"/>
       <c r="D46" s="9" t="inlineStr"/>
       <c r="E46" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>Pack Of 4 Medoviks And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="4" t="inlineStr"/>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="9" t="inlineStr"/>
+      <c r="E47" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="4" t="inlineStr"/>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="9" t="inlineStr"/>
+      <c r="E48" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G46" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr"/>
-      <c r="D47" s="6" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Pack Of 9 Medoviks And 6 Macarons</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>MH-MUM-Express Outlet Jio World</t>
         </is>
       </c>
-      <c r="E47" s="5" t="n">
+      <c r="E49" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F49" s="7" t="inlineStr">
         <is>
           <t>Italian Tiramisu Medovik With Macaron</t>
         </is>
       </c>
-      <c r="G47" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>MH-MUM-Express Outlet Palladium</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>Italian Cappuccino</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>PUN</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>MH-PUN-Cloud FC Tathewadi</t>
         </is>
       </c>
-      <c r="E48" s="5" t="n">
+      <c r="E51" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F51" s="7" t="inlineStr">
         <is>
           <t>Harley's Special Mawa Bar Cake (250 Gms)</t>
         </is>
       </c>
-      <c r="G48" s="8" t="inlineStr">
+      <c r="G51" s="8" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
@@ -2096,7 +2195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2117,12 +2216,12 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Total Outlets: 5</t>
+          <t>Total Outlets: 7</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Still OUT: 7</t>
+          <t>Still OUT: 11</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
@@ -2242,43 +2341,49 @@
       <c r="C5" s="4" t="inlineStr"/>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>KA-BLR-Cloud FC Malleshwaram</t>
+          <t>KA-BLR-Cloud FC Basaveshwara Nagar</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Assorted Cheesecakes (Pack Of 6)</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
+          <t>Assorted French Macarons (Pack Of 5)</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="4" t="inlineStr"/>
+      <c r="A6" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Cloud FC Electronic City</t>
+        </is>
+      </c>
       <c r="E6" s="5" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
+          <t>Signature Belgium Chocolate Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
         </is>
       </c>
     </row>
@@ -2292,68 +2397,68 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="9" t="inlineStr"/>
       <c r="E7" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
+          <t>Danish Hazelnut Chocolate Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Pack Of 4 Medoviks And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Cloud FC Malleshwaram</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
         <is>
           <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Cloud FC NBL</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Medoviks And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="9" t="inlineStr"/>
-      <c r="E9" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
         </is>
       </c>
     </row>
@@ -2367,16 +2472,16 @@
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="9" t="inlineStr"/>
       <c r="E10" s="5" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 5)</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Italian Tiramisu Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -2390,22 +2495,22 @@
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="9" t="inlineStr"/>
       <c r="E11" s="5" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
@@ -2415,15 +2520,15 @@
       <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>KA-BLR-Cloud FC Whitefield</t>
+          <t>KA-BLR-Cloud FC NBL</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
+          <t>Pack Of 4 Medoviks And 4 Macarons</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -2433,31 +2538,25 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="4" t="n">
-        <v>5</v>
-      </c>
+      <c r="A13" s="4" t="inlineStr"/>
       <c r="B13" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Ivory Lounge JP Nagar</t>
-        </is>
-      </c>
+      <c r="D13" s="9" t="inlineStr"/>
       <c r="E13" s="5" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 5)</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
         </is>
       </c>
     </row>
@@ -2471,14 +2570,118 @@
       <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="9" t="inlineStr"/>
       <c r="E14" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 5)</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="4" t="inlineStr"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="9" t="inlineStr"/>
+      <c r="E15" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Cloud FC Sarjapur</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Ivory Lounge JP Nagar</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 5)</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="9" t="inlineStr"/>
+      <c r="E18" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>Assorted French Macarons (Pack Of 12)</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
@@ -2495,7 +2698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2521,7 +2724,7 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Still OUT: 9</t>
+          <t>Still OUT: 8</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
@@ -2593,11 +2796,11 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Assorted Cheesecakes (Pack Of 6)</t>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -2616,63 +2819,63 @@
       <c r="C4" s="4" t="inlineStr"/>
       <c r="D4" s="9" t="inlineStr"/>
       <c r="E4" s="5" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
+          <t>Lotus Biscoff Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>TG-HYD-Cloud FC Charminar</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr"/>
+      <c r="E6" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
           <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="4" t="inlineStr"/>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="9" t="inlineStr"/>
-      <c r="E5" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Lotus Biscoff Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Cloud FC Charminar</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -2691,11 +2894,11 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="9" t="inlineStr"/>
       <c r="E7" s="5" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+          <t>Lotus Biscoff Cheesecake With Macaron</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -2714,11 +2917,11 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="9" t="inlineStr"/>
       <c r="E8" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Lotus Biscoff Cheesecake With Macaron</t>
+          <t>Assorted Cheesecakes (Pack Of 12)</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -2728,49 +2931,49 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="9" t="inlineStr"/>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>TG-HYD-Cloud FC Habsiguda</t>
+        </is>
+      </c>
       <c r="E9" s="5" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Assorted Cheesecakes (Pack Of 12)</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="4" t="n">
-        <v>3</v>
-      </c>
+      <c r="A10" s="4" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Cloud FC Habsiguda</t>
-        </is>
-      </c>
+      <c r="D10" s="9" t="inlineStr"/>
       <c r="E10" s="5" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -2789,11 +2992,11 @@
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="9" t="inlineStr"/>
       <c r="E11" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Assorted Cheesecakes (Pack Of 6)</t>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -2803,31 +3006,37 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="4" t="inlineStr"/>
+      <c r="A12" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="9" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>TG-HYD-Express Outlet Madhapur</t>
+        </is>
+      </c>
       <c r="E12" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Italian Tiramisu Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
@@ -2837,26 +3046,26 @@
       <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>TG-HYD-Express Outlet Madhapur</t>
+          <t>TG-HYD-Express Outlet Manikonda</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
@@ -2866,70 +3075,41 @@
       <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>TG-HYD-Express Outlet Manikonda</t>
+          <t>TG-HYD-Express Outlet Sainikpuri</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
+          <t>Assorted French Macarons (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="4" t="inlineStr"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="9" t="inlineStr"/>
+      <c r="E15" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
           <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Express Outlet Sainikpuri</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
-        </is>
-      </c>
       <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="9" t="inlineStr"/>
-      <c r="E16" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
@@ -2967,7 +3147,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Total Outlets: 2</t>
+          <t>Total Outlets: 5</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
@@ -3040,32 +3220,38 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
+          <t>MH-MUM-Cloud FC BKC</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 24)</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
           <t>MH-MUM-Cloud FC Borivali</t>
         </is>
       </c>
-      <c r="E3" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Medoviks And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="4" t="inlineStr"/>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="9" t="inlineStr"/>
       <c r="E4" s="5" t="n">
         <v>4</v>
       </c>
@@ -3104,20 +3290,26 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="4" t="inlineStr"/>
+      <c r="A6" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>MH-MUM-Cloud FC Chembur</t>
+        </is>
+      </c>
       <c r="E6" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Signature Belgium Chocolate Medovik With Macaron</t>
+          <t>Assorted French Macarons (Pack Of 5)</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -3136,11 +3328,11 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="9" t="inlineStr"/>
       <c r="E7" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
+          <t>Assorted French Macarons (Pack Of 12)</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -3159,11 +3351,11 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="9" t="inlineStr"/>
       <c r="E8" s="5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Danish Hazelnut Chocolate Medovik With Macaron</t>
+          <t>Pack Of 4 Medoviks And 4 Macarons</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -3182,11 +3374,11 @@
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="9" t="inlineStr"/>
       <c r="E9" s="5" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -3205,11 +3397,11 @@
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="9" t="inlineStr"/>
       <c r="E10" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Harley's Spl. Classic Russian Medovik With Macaron</t>
+          <t>Pack Of 9 Medoviks And 6 Macarons</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -3219,20 +3411,26 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="4" t="inlineStr"/>
+      <c r="A11" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="9" t="inlineStr"/>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>MH-MUM-Express Outlet Jio World</t>
+        </is>
+      </c>
       <c r="E11" s="5" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+          <t>Italian Tiramisu Medovik With Macaron</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -3243,7 +3441,7 @@
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
@@ -3253,15 +3451,15 @@
       <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>MH-MUM-Express Outlet Jio World</t>
+          <t>MH-MUM-Express Outlet Palladium</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
+          <t>Italian Cappuccino</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Filter Morning/Evening OOS by active outlets in daily CSV; add NCR and remove stale screenshots
</commit_message>
<xml_diff>
--- a/Oct - 05/Evening/Evening_OOS_Summary_2026-10-05.xlsx
+++ b/Oct - 05/Evening/Evening_OOS_Summary_2026-10-05.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -542,17 +542,17 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Total Outlets: 21</t>
+          <t>Total Outlets: 19</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Still OUT: 34</t>
+          <t>Still OUT: 23</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Restored IN: 15</t>
+          <t>Restored IN: 27</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
@@ -849,9 +849,9 @@
           <t>Signature Belgium Chocolate Medovik With Macaron</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -872,9 +872,9 @@
           <t>Danish Hazelnut Chocolate Medovik With Macaron</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>KA-BLR-Cloud FC Basaveshwara Nagar</t>
+          <t>KA-BLR-Cloud FC Bellandur</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
@@ -898,41 +898,35 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 5)</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="n">
-        <v>5</v>
-      </c>
+      <c r="A15" s="4" t="inlineStr"/>
       <c r="B15" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Cloud FC Electronic City</t>
-        </is>
-      </c>
+      <c r="D15" s="9" t="inlineStr"/>
       <c r="E15" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Signature Belgium Chocolate Medovik With Macaron</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Assorted Medoviks (Pack Of 6)</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -946,16 +940,16 @@
       <c r="C16" s="4" t="inlineStr"/>
       <c r="D16" s="9" t="inlineStr"/>
       <c r="E16" s="5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Danish Hazelnut Chocolate Medovik With Macaron</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -969,63 +963,63 @@
       <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="9" t="inlineStr"/>
       <c r="E17" s="5" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
+          <t>Harley's Signatures (Pack of 8)</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="9" t="inlineStr"/>
+      <c r="E18" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
           <t>Pack Of 4 Medoviks And 4 Macarons</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>KA-BLR-Cloud FC Malleshwaram</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E19" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>Assorted Cheesecakes (Pack Of 6)</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="4" t="inlineStr"/>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr"/>
-      <c r="D19" s="9" t="inlineStr"/>
-      <c r="E19" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -1044,143 +1038,149 @@
       <c r="C20" s="4" t="inlineStr"/>
       <c r="D20" s="9" t="inlineStr"/>
       <c r="E20" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Italian Tiramisu Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="4" t="inlineStr"/>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr"/>
+      <c r="D21" s="9" t="inlineStr"/>
+      <c r="E21" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="4" t="n">
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr"/>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Cloud FC Nagawara</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr"/>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Cloud FC NBL</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Medoviks And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="4" t="inlineStr"/>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="9" t="inlineStr"/>
-      <c r="E22" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="4" t="inlineStr"/>
       <c r="B23" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr"/>
-      <c r="D23" s="9" t="inlineStr"/>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Cloud FC Whitefield</t>
+        </is>
+      </c>
       <c r="E23" s="5" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
+          <t>Assorted French Macarons (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Ivory Lounge JP Nagar</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
           <t>Assorted French Macarons (Pack Of 5)</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="4" t="inlineStr"/>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="9" t="inlineStr"/>
-      <c r="E24" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="9" t="inlineStr"/>
+      <c r="E25" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>Assorted French Macarons (Pack Of 12)</t>
         </is>
       </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr"/>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Cloud FC Sarjapur</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -1193,23 +1193,27 @@
           <t>2026/10/05</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>HYD</t>
+        </is>
+      </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>KA-BLR-Ivory Lounge JP Nagar</t>
+          <t>TG-HYD-Cloud FC Attapur</t>
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 5)</t>
-        </is>
-      </c>
-      <c r="G26" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
         </is>
       </c>
     </row>
@@ -1223,90 +1227,80 @@
       <c r="C27" s="4" t="inlineStr"/>
       <c r="D27" s="9" t="inlineStr"/>
       <c r="E27" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
-        </is>
-      </c>
-      <c r="G27" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="4" t="n">
+      <c r="A28" s="4" t="inlineStr"/>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="9" t="inlineStr"/>
+      <c r="E28" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>Lotus Biscoff Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>HYD</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Cloud FC Attapur</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G28" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="4" t="inlineStr"/>
       <c r="B29" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr"/>
-      <c r="D29" s="9" t="inlineStr"/>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>TG-HYD-Cloud FC Charminar</t>
+        </is>
+      </c>
       <c r="E29" s="5" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Lotus Biscoff Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="4" t="n">
-        <v>11</v>
-      </c>
+      <c r="A30" s="4" t="inlineStr"/>
       <c r="B30" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Cloud FC Charminar</t>
-        </is>
-      </c>
+      <c r="D30" s="9" t="inlineStr"/>
       <c r="E30" s="5" t="n">
         <v>9</v>
       </c>
@@ -1392,7 +1386,7 @@
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
@@ -1467,7 +1461,7 @@
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
@@ -1477,15 +1471,15 @@
       <c r="C37" s="4" t="inlineStr"/>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>TG-HYD-Express Outlet Madhapur</t>
+          <t>TG-HYD-Express Outlet Kapil Tower</t>
         </is>
       </c>
       <c r="E37" s="5" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
         </is>
       </c>
       <c r="G37" s="10" t="inlineStr">
@@ -1496,7 +1490,7 @@
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
@@ -1506,26 +1500,26 @@
       <c r="C38" s="4" t="inlineStr"/>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>TG-HYD-Express Outlet Manikonda</t>
+          <t>TG-HYD-Express Outlet Madhapur</t>
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G38" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Italian Tiramisu Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G38" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
@@ -1535,38 +1529,44 @@
       <c r="C39" s="4" t="inlineStr"/>
       <c r="D39" s="6" t="inlineStr">
         <is>
+          <t>TG-HYD-Express Outlet Manikonda</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr"/>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
           <t>TG-HYD-Express Outlet Sainikpuri</t>
         </is>
       </c>
-      <c r="E39" s="5" t="n">
+      <c r="E40" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>Assorted French Macarons (Pack Of 12)</t>
-        </is>
-      </c>
-      <c r="G39" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="4" t="inlineStr"/>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="9" t="inlineStr"/>
-      <c r="E40" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -1591,15 +1591,15 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>MH-MUM-Cloud FC BKC</t>
+          <t>MH-MUM-Cloud FC Borivali</t>
         </is>
       </c>
       <c r="E41" s="5" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 24)</t>
+          <t>Pack Of 4 Medoviks And 4 Macarons</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
@@ -1609,20 +1609,14 @@
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="4" t="n">
-        <v>17</v>
-      </c>
+      <c r="A42" s="4" t="inlineStr"/>
       <c r="B42" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr"/>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>MH-MUM-Cloud FC Borivali</t>
-        </is>
-      </c>
+      <c r="D42" s="9" t="inlineStr"/>
       <c r="E42" s="5" t="n">
         <v>4</v>
       </c>
@@ -1661,26 +1655,20 @@
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="4" t="n">
-        <v>18</v>
-      </c>
+      <c r="A44" s="4" t="inlineStr"/>
       <c r="B44" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr"/>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>MH-MUM-Cloud FC Chembur</t>
-        </is>
-      </c>
+      <c r="D44" s="9" t="inlineStr"/>
       <c r="E44" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 5)</t>
+          <t>Signature Belgium Chocolate Medovik With Macaron</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
@@ -1699,11 +1687,11 @@
       <c r="C45" s="4" t="inlineStr"/>
       <c r="D45" s="9" t="inlineStr"/>
       <c r="E45" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
+          <t>Italian Tiramisu Medovik With Macaron</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
@@ -1722,11 +1710,11 @@
       <c r="C46" s="4" t="inlineStr"/>
       <c r="D46" s="9" t="inlineStr"/>
       <c r="E46" s="5" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>Pack Of 4 Medoviks And 4 Macarons</t>
+          <t>Danish Hazelnut Chocolate Medovik With Macaron</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
@@ -1745,11 +1733,11 @@
       <c r="C47" s="4" t="inlineStr"/>
       <c r="D47" s="9" t="inlineStr"/>
       <c r="E47" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
       <c r="G47" s="8" t="inlineStr">
@@ -1768,40 +1756,34 @@
       <c r="C48" s="4" t="inlineStr"/>
       <c r="D48" s="9" t="inlineStr"/>
       <c r="E48" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Harley's Spl. Classic Russian Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="4" t="inlineStr"/>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="9" t="inlineStr"/>
+      <c r="E49" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 9 Medoviks And 6 Macarons</t>
-        </is>
-      </c>
-      <c r="G48" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr"/>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>MH-MUM-Express Outlet Jio World</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="n">
-        <v>9</v>
-      </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
@@ -1812,7 +1794,7 @@
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
@@ -1822,15 +1804,15 @@
       <c r="C50" s="4" t="inlineStr"/>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>MH-MUM-Express Outlet Palladium</t>
+          <t>MH-MUM-Express Outlet Jio World</t>
         </is>
       </c>
       <c r="E50" s="5" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>Italian Cappuccino</t>
+          <t>Italian Tiramisu Medovik With Macaron</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
@@ -1841,7 +1823,7 @@
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
@@ -1867,6 +1849,35 @@
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr"/>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>MH-PUN-Express Outlet Vimannagar</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>Italian Tiramisu Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
@@ -2195,7 +2206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2216,17 +2227,17 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Total Outlets: 7</t>
+          <t>Total Outlets: 6</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Still OUT: 11</t>
+          <t>Still OUT: 0</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Restored IN: 5</t>
+          <t>Restored IN: 14</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
@@ -2300,9 +2311,9 @@
           <t>Signature Belgium Chocolate Medovik With Macaron</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -2323,9 +2334,9 @@
           <t>Danish Hazelnut Chocolate Medovik With Macaron</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2352,7 @@
       <c r="C5" s="4" t="inlineStr"/>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>KA-BLR-Cloud FC Basaveshwara Nagar</t>
+          <t>KA-BLR-Cloud FC Bellandur</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
@@ -2349,41 +2360,35 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 5)</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="4" t="n">
-        <v>3</v>
-      </c>
+      <c r="A6" s="4" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Cloud FC Electronic City</t>
-        </is>
-      </c>
+      <c r="D6" s="9" t="inlineStr"/>
       <c r="E6" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Signature Belgium Chocolate Medovik With Macaron</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Assorted Medoviks (Pack Of 6)</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -2397,16 +2402,16 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="9" t="inlineStr"/>
       <c r="E7" s="5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Danish Hazelnut Chocolate Medovik With Macaron</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -2420,63 +2425,63 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="9" t="inlineStr"/>
       <c r="E8" s="5" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
+          <t>Harley's Signatures (Pack of 8)</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr"/>
+      <c r="E9" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
           <t>Pack Of 4 Medoviks And 4 Macarons</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Cloud FC Malleshwaram</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Cloud FC Malleshwaram</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Assorted Cheesecakes (Pack Of 6)</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="4" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="9" t="inlineStr"/>
-      <c r="E10" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -2495,193 +2500,147 @@
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="9" t="inlineStr"/>
       <c r="E11" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Italian Tiramisu Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr"/>
+      <c r="E12" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="4" t="n">
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Cloud FC Nagawara</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Cloud FC NBL</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Medoviks And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="9" t="inlineStr"/>
-      <c r="E13" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="4" t="inlineStr"/>
       <c r="B14" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="9" t="inlineStr"/>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Cloud FC Whitefield</t>
+        </is>
+      </c>
       <c r="E14" s="5" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
+          <t>Assorted French Macarons (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>KA-BLR-Ivory Lounge JP Nagar</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
           <t>Assorted French Macarons (Pack Of 5)</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="inlineStr"/>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="9" t="inlineStr"/>
-      <c r="E15" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="9" t="inlineStr"/>
+      <c r="E16" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>Assorted French Macarons (Pack Of 12)</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Cloud FC Sarjapur</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>KA-BLR-Ivory Lounge JP Nagar</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>Assorted French Macarons (Pack Of 5)</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="9" t="inlineStr"/>
-      <c r="E18" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G16" s="10" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
@@ -2698,7 +2657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2719,17 +2678,17 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Total Outlets: 6</t>
+          <t>Total Outlets: 7</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Still OUT: 8</t>
+          <t>Still OUT: 7</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Restored IN: 5</t>
+          <t>Restored IN: 8</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
@@ -2796,11 +2755,11 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -2819,63 +2778,63 @@
       <c r="C4" s="4" t="inlineStr"/>
       <c r="D4" s="9" t="inlineStr"/>
       <c r="E4" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="9" t="inlineStr"/>
+      <c r="E5" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Lotus Biscoff Cheesecake With Macaron</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="4" t="n">
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>TG-HYD-Cloud FC Charminar</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="4" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
       <c r="E6" s="5" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -2894,11 +2853,11 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="9" t="inlineStr"/>
       <c r="E7" s="5" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Lotus Biscoff Cheesecake With Macaron</t>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -2917,11 +2876,11 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="9" t="inlineStr"/>
       <c r="E8" s="5" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Assorted Cheesecakes (Pack Of 12)</t>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -2931,31 +2890,25 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="4" t="n">
-        <v>3</v>
-      </c>
+      <c r="A9" s="4" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Cloud FC Habsiguda</t>
-        </is>
-      </c>
+      <c r="D9" s="9" t="inlineStr"/>
       <c r="E9" s="5" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Lotus Biscoff Cheesecake With Macaron</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -2969,88 +2922,82 @@
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="9" t="inlineStr"/>
       <c r="E10" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Assorted Cheesecakes (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>TG-HYD-Cloud FC Habsiguda</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr"/>
+      <c r="E12" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Assorted Cheesecakes (Pack Of 6)</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="5" t="n">
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr"/>
+      <c r="E13" s="5" t="n">
         <v>18</v>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Express Outlet Madhapur</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>TG-HYD-Express Outlet Manikonda</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>15</v>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
@@ -3065,7 +3012,7 @@
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
@@ -3075,41 +3022,105 @@
       <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>TG-HYD-Express Outlet Sainikpuri</t>
+          <t>TG-HYD-Express Outlet Kapil Tower</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
+          <t>Assorted Cheesecakes (Pack Of 6)</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="inlineStr"/>
+      <c r="A15" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="9" t="inlineStr"/>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>TG-HYD-Express Outlet Madhapur</t>
+        </is>
+      </c>
       <c r="E15" s="5" t="n">
         <v>19</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
+          <t>Italian Tiramisu Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>TG-HYD-Express Outlet Manikonda</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
           <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>TG-HYD-Express Outlet Sainikpuri</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Assorted French Macarons (Pack Of 12)</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
@@ -3147,7 +3158,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Total Outlets: 5</t>
+          <t>Total Outlets: 2</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
@@ -3220,15 +3231,15 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>MH-MUM-Cloud FC BKC</t>
+          <t>MH-MUM-Cloud FC Borivali</t>
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 24)</t>
+          <t>Pack Of 4 Medoviks And 4 Macarons</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -3238,20 +3249,14 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="A4" s="4" t="inlineStr"/>
       <c r="B4" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>MH-MUM-Cloud FC Borivali</t>
-        </is>
-      </c>
+      <c r="D4" s="9" t="inlineStr"/>
       <c r="E4" s="5" t="n">
         <v>4</v>
       </c>
@@ -3290,26 +3295,20 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="4" t="n">
-        <v>3</v>
-      </c>
+      <c r="A6" s="4" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
           <t>2026/10/05</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>MH-MUM-Cloud FC Chembur</t>
-        </is>
-      </c>
+      <c r="D6" s="9" t="inlineStr"/>
       <c r="E6" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 5)</t>
+          <t>Signature Belgium Chocolate Medovik With Macaron</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -3328,11 +3327,11 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="9" t="inlineStr"/>
       <c r="E7" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Assorted French Macarons (Pack Of 12)</t>
+          <t>Italian Tiramisu Medovik With Macaron</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -3351,11 +3350,11 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="9" t="inlineStr"/>
       <c r="E8" s="5" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Pack Of 4 Medoviks And 4 Macarons</t>
+          <t>Danish Hazelnut Chocolate Medovik With Macaron</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -3374,11 +3373,11 @@
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="9" t="inlineStr"/>
       <c r="E9" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
+          <t>Chef's Favourite Blueberry Cheesecake With Macaron</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -3397,40 +3396,34 @@
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="9" t="inlineStr"/>
       <c r="E10" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Harley's Spl. Classic Russian Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr"/>
+      <c r="E11" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Pack Of 9 Medoviks And 6 Macarons</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>2026/10/05</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>MH-MUM-Express Outlet Jio World</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>9</v>
-      </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Italian Tiramisu Medovik With Macaron</t>
+          <t>Pack Of 4 Cheesecakes And 4 Macarons</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -3441,7 +3434,7 @@
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
@@ -3451,15 +3444,15 @@
       <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>MH-MUM-Express Outlet Palladium</t>
+          <t>MH-MUM-Express Outlet Jio World</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Italian Cappuccino</t>
+          <t>Italian Tiramisu Medovik With Macaron</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -3479,7 +3472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3500,12 +3493,12 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Total Outlets: 1</t>
+          <t>Total Outlets: 2</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Still OUT: 1</t>
+          <t>Still OUT: 2</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
@@ -3585,6 +3578,35 @@
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>MH-PUN-Express Outlet Vimannagar</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Italian Tiramisu Medovik With Macaron</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>

</xml_diff>